<commit_message>
Phase 3: re-add breadboard kit, note why the multimeter is a must-have
Hasan asked for breadboards and wires. Kimi had marked the kit optional (the
ESP32 dev board + Dupont + WAGO cover prototyping), but it is C$19.99 and the
budget has room, so it's back (B0BMFXPSVG, 830 + 400 point + jumpers).

A friend of Hasan's warned that without a multimeter things get blown up. It is
already in the cart (B07H65J7DQ, C$19.98). Its note now gives the reason: check
each adjustable PSU before plugging servos in, since 12 V by mistake burns the
6 V MG996R hand servos.

Cart: 29 items, C$390.17 pre-tax, about C$441 with HST. Nothing ordered.
</commit_message>
<xml_diff>
--- a/robotai_BOM.xlsx
+++ b/robotai_BOM.xlsx
@@ -2768,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2790,7 +2790,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Checked with Kimi (senior build manager) on 2026-09-27: cut the crimper and breadboard, swapped the wrench set for one 13 mm wrench, added nylock nuts, files, sandpaper, knife, tweezers, fuses, switch.</t>
+          <t>Checked with Kimi (senior build manager) on 2026-09-27: cut the crimper and breadboard, swapped the wrench set for one 13 mm wrench, added nylock nuts, files, sandpaper, knife, tweezers, fuses, switch. Breadboard kit re-added at Hasan's request (Kimi had marked it optional).</t>
         </is>
       </c>
     </row>
@@ -3403,28 +3403,28 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Check PSU voltage before plugging servos in.</t>
+          <t>Must-have: check each power supply's voltage before plugging servos in (12 V by mistake burns 6 V servos).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Heat shrink</t>
+          <t>Breadboards + jumper wires</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ASHINER heat shrink kit, 580 pcs</t>
+          <t>830 + 400 point breadboards with jumper wire kit</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B08XXGNJHG</t>
+          <t>https://www.amazon.ca/dp/B0BMFXPSVG</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>14.99</v>
+        <v>19.99</v>
       </c>
       <c r="E23" s="12" t="n">
         <v>1</v>
@@ -3435,28 +3435,28 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Covers solder joints.</t>
+          <t>Test sensors/servo signals before soldering. Kimi said optional; re-added because Hasan asked.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Calipers</t>
+          <t>Heat shrink</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>ADORIC digital caliper 0-150 mm</t>
+          <t>ASHINER heat shrink kit, 580 pcs</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07DFFYCXS</t>
+          <t>https://www.amazon.ca/dp/B08XXGNJHG</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>11.43</v>
+        <v>14.99</v>
       </c>
       <c r="E24" s="12" t="n">
         <v>1</v>
@@ -3467,28 +3467,28 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Measure screws and printed parts.</t>
+          <t>Covers solder joints.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Zip ties</t>
+          <t>Calipers</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>400 assorted zip ties</t>
+          <t>ADORIC digital caliper 0-150 mm</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B08TVLYB3Q</t>
+          <t>https://www.amazon.ca/dp/B07DFFYCXS</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>11.98</v>
+        <v>11.43</v>
       </c>
       <c r="E25" s="12" t="n">
         <v>1</v>
@@ -3499,28 +3499,28 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Cable management.</t>
+          <t>Measure screws and printed parts.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Hot glue</t>
+          <t>Zip ties</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Surebonder LT-160 mini glue gun</t>
+          <t>400 assorted zip ties</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B004BPPHYE</t>
+          <t>https://www.amazon.ca/dp/B08TVLYB3Q</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>7.47</v>
+        <v>11.98</v>
       </c>
       <c r="E26" s="12" t="n">
         <v>1</v>
@@ -3531,28 +3531,28 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>InMoov wire management method.</t>
+          <t>Cable management.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Needle files</t>
+          <t>Hot glue</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>10-piece needle file set</t>
+          <t>Surebonder LT-160 mini glue gun</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07PPYWSCY</t>
+          <t>https://www.amazon.ca/dp/B004BPPHYE</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>9.99</v>
+        <v>7.47</v>
       </c>
       <c r="E27" s="12" t="n">
         <v>1</v>
@@ -3563,28 +3563,28 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Fit printed parts (ball races, pistons). Kimi: day-1 blocker.</t>
+          <t>InMoov wire management method.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Sandpaper</t>
+          <t>Needle files</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>3M sandpaper 100/150/220 grit, 5 sheets</t>
+          <t>10-piece needle file set</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B00004Z48U</t>
+          <t>https://www.amazon.ca/dp/B07PPYWSCY</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>7.97</v>
+        <v>9.99</v>
       </c>
       <c r="E28" s="12" t="n">
         <v>1</v>
@@ -3595,28 +3595,28 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Smooth printed parts.</t>
+          <t>Fit printed parts (ball races, pistons). Kimi: day-1 blocker.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Hobby knife</t>
+          <t>Sandpaper</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>VViViD modelers knife + spare blades</t>
+          <t>3M sandpaper 100/150/220 grit, 5 sheets</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0CL5F9M4H</t>
+          <t>https://www.amazon.ca/dp/B00004Z48U</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>7.98</v>
+        <v>7.97</v>
       </c>
       <c r="E29" s="12" t="n">
         <v>1</v>
@@ -3627,28 +3627,28 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Clean up prints.</t>
+          <t>Smooth printed parts.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Tweezers</t>
+          <t>Hobby knife</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>NARZ 4-piece tweezers</t>
+          <t>VViViD modelers knife + spare blades</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B09JLXKWB5</t>
+          <t>https://www.amazon.ca/dp/B0CL5F9M4H</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>6.29</v>
+        <v>7.98</v>
       </c>
       <c r="E30" s="12" t="n">
         <v>1</v>
@@ -3659,28 +3659,28 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Threading finger tendons.</t>
+          <t>Clean up prints.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Safety glasses</t>
+          <t>Tweezers</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Clear safety glasses, 3-pack</t>
+          <t>NARZ 4-piece tweezers</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0F2JL22QN</t>
+          <t>https://www.amazon.ca/dp/B09JLXKWB5</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>13.49</v>
+        <v>6.29</v>
       </c>
       <c r="E31" s="12" t="n">
         <v>1</v>
@@ -3691,30 +3691,46 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
+          <t>Threading finger tendons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Safety glasses</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Clear safety glasses, 3-pack</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0F2JL22QN</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="13">
+        <f>D32*E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
           <t>For cutting, soldering, springs.</t>
         </is>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
-        <is>
-          <t>Subtotal (CAD, pre-tax)</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="16">
-        <f>SUM(F5:F31)</f>
-        <v/>
-      </c>
-      <c r="G32" s="15" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>With HST 13%</t>
+          <t>Subtotal (CAD, pre-tax)</t>
         </is>
       </c>
       <c r="B33" s="15" t="n"/>
@@ -3722,14 +3738,30 @@
       <c r="D33" s="15" t="n"/>
       <c r="E33" s="15" t="n"/>
       <c r="F33" s="16">
-        <f>F32*1.13</f>
+        <f>SUM(F5:F32)</f>
         <v/>
       </c>
       <c r="G33" s="15" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>With HST 13%</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="16">
+        <f>F33*1.13</f>
+        <v/>
+      </c>
+      <c r="G34" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A33:E33"/>
   </mergeCells>
   <hyperlinks>
@@ -3760,6 +3792,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Phase 3: add the DC barrel adapters that were never ordered
Hasan asked whether anything else was missing. I compared every Phase 1 core
line against the Amazon.ca order history (ESP32, MG996R x12, PCA9685, 2x
SHNITPWR, PE braid, springs, Dupont, 18 AWG wire all present). One gap: the
5.5x2.1 mm DC barrel-to-screw-terminal adapters (B0C4JJ2HB4) were planned but
never bought. Without them the power supplies can't be wired to the PCA9685
V+ terminals without cutting the plugs off. Added at C$11.99.

Cart: 30 items, C$402.16 pre-tax, about C$454 with HST. Nothing ordered.
</commit_message>
<xml_diff>
--- a/robotai_BOM.xlsx
+++ b/robotai_BOM.xlsx
@@ -2768,7 +2768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2790,7 +2790,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Checked with Kimi (senior build manager) on 2026-09-27: cut the crimper and breadboard, swapped the wrench set for one 13 mm wrench, added nylock nuts, files, sandpaper, knife, tweezers, fuses, switch. Breadboard kit re-added at Hasan's request (Kimi had marked it optional).</t>
+          <t>Checked with Kimi (senior build manager) on 2026-09-27: cut the crimper and breadboard, swapped the wrench set for one 13 mm wrench, added nylock nuts, files, sandpaper, knife, tweezers, fuses, switch. Breadboard kit re-added at Hasan's request (Kimi had marked it optional). Recheck vs orders: the DC barrel-to-screw adapters from Phase 1 were never ordered; added.</t>
         </is>
       </c>
     </row>
@@ -3090,21 +3090,21 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Wire joiners</t>
+          <t>Power plug adapters (PSU to boards)</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>WAGO 221 lever connectors, 25 pcs</t>
+          <t>20 pcs 5.5 x 2.1 mm DC barrel to screw terminal</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0BYBHYLG2</t>
+          <t>https://www.amazon.ca/dp/B0C4JJ2HB4</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
-        <v>29.39</v>
+        <v>11.99</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>1</v>
@@ -3115,28 +3115,28 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Join power wires without soldering.</t>
+          <t>Was in the Phase 1 plan but never ordered. Connects the 2 power supplies to the PCA9685 servo boards.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Fuses</t>
+          <t>Wire joiners</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>12 AWG inline fuse holders, 4 pcs</t>
+          <t>WAGO 221 lever connectors, 25 pcs</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0FDJYRGB7</t>
+          <t>https://www.amazon.ca/dp/B0BYBHYLG2</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>9.99</v>
+        <v>29.39</v>
       </c>
       <c r="E14" s="12" t="n">
         <v>1</v>
@@ -3147,28 +3147,28 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>10 A fuse on each power supply line.</t>
+          <t>Join power wires without soldering.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Main power switch</t>
+          <t>Fuses</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Nilight rocker switch 20 A</t>
+          <t>12 AWG inline fuse holders, 4 pcs</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B06ZZHX6K3</t>
+          <t>https://www.amazon.ca/dp/B0FDJYRGB7</t>
         </is>
       </c>
       <c r="D15" s="11" t="n">
-        <v>4.62</v>
+        <v>9.99</v>
       </c>
       <c r="E15" s="12" t="n">
         <v>1</v>
@@ -3179,28 +3179,28 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>One switch kills servo power.</t>
+          <t>10 A fuse on each power supply line.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Screwdrivers</t>
+          <t>Main power switch</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>STREBITO 124-piece precision screwdriver set</t>
+          <t>Nilight rocker switch 20 A</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0968D5PSC</t>
+          <t>https://www.amazon.ca/dp/B06ZZHX6K3</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>25.99</v>
+        <v>4.62</v>
       </c>
       <c r="E16" s="12" t="n">
         <v>1</v>
@@ -3211,28 +3211,28 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Phillips PH0-PH2 + hex bits for M2-M4 screws.</t>
+          <t>One switch kills servo power.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Hex keys</t>
+          <t>Screwdrivers</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>GEARWRENCH 9-piece metric ball-end hex keys</t>
+          <t>STREBITO 124-piece precision screwdriver set</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B098TYMJ3X</t>
+          <t>https://www.amazon.ca/dp/B0968D5PSC</t>
         </is>
       </c>
       <c r="D17" s="11" t="n">
-        <v>10.99</v>
+        <v>25.99</v>
       </c>
       <c r="E17" s="12" t="n">
         <v>1</v>
@@ -3243,28 +3243,28 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>1.5-10 mm. Your countersunk kit: 2 mm = M3, 2.5 mm = M4. 6 mm = the M8 bolts.</t>
+          <t>Phillips PH0-PH2 + hex bits for M2-M4 screws.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Pliers + cutter</t>
+          <t>Hex keys</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>SPEEDWOX mini long-nose pliers with cutter</t>
+          <t>GEARWRENCH 9-piece metric ball-end hex keys</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0CGHRCHP5</t>
+          <t>https://www.amazon.ca/dp/B098TYMJ3X</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>9.69</v>
+        <v>10.99</v>
       </c>
       <c r="E18" s="12" t="n">
         <v>1</v>
@@ -3275,28 +3275,28 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Cheap single tool: grip + snip.</t>
+          <t>1.5-10 mm. Your countersunk kit: 2 mm = M3, 2.5 mm = M4. 6 mm = the M8 bolts.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Wire stripper</t>
+          <t>Pliers + cutter</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Solsop self-adjusting wire stripper</t>
+          <t>SPEEDWOX mini long-nose pliers with cutter</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07XXMLFMV</t>
+          <t>https://www.amazon.ca/dp/B0CGHRCHP5</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>10.19</v>
+        <v>9.69</v>
       </c>
       <c r="E19" s="12" t="n">
         <v>1</v>
@@ -3307,28 +3307,28 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Strips 10-24 AWG.</t>
+          <t>Cheap single tool: grip + snip.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Soldering iron</t>
+          <t>Wire stripper</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>60 W adjustable soldering iron kit</t>
+          <t>Solsop self-adjusting wire stripper</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B08K8VFTF9</t>
+          <t>https://www.amazon.ca/dp/B07XXMLFMV</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
-        <v>13.99</v>
+        <v>10.19</v>
       </c>
       <c r="E20" s="12" t="n">
         <v>1</v>
@@ -3339,28 +3339,28 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Cheapest decent kit (446 reviews).</t>
+          <t>Strips 10-24 AWG.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Solder</t>
+          <t>Soldering iron</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>TOWOT 63/37 rosin-core solder 0.8 mm</t>
+          <t>60 W adjustable soldering iron kit</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0943TPRXK</t>
+          <t>https://www.amazon.ca/dp/B08K8VFTF9</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>12.97</v>
+        <v>13.99</v>
       </c>
       <c r="E21" s="12" t="n">
         <v>1</v>
@@ -3371,28 +3371,28 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>0.8 mm wire, easy for beginners.</t>
+          <t>Cheapest decent kit (446 reviews).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Multimeter</t>
+          <t>Solder</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Digital multimeter</t>
+          <t>TOWOT 63/37 rosin-core solder 0.8 mm</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07H65J7DQ</t>
+          <t>https://www.amazon.ca/dp/B0943TPRXK</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
-        <v>19.98</v>
+        <v>12.97</v>
       </c>
       <c r="E22" s="12" t="n">
         <v>1</v>
@@ -3403,28 +3403,28 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Must-have: check each power supply's voltage before plugging servos in (12 V by mistake burns 6 V servos).</t>
+          <t>0.8 mm wire, easy for beginners.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Breadboards + jumper wires</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>830 + 400 point breadboards with jumper wire kit</t>
+          <t>Digital multimeter</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0BMFXPSVG</t>
+          <t>https://www.amazon.ca/dp/B07H65J7DQ</t>
         </is>
       </c>
       <c r="D23" s="11" t="n">
-        <v>19.99</v>
+        <v>19.98</v>
       </c>
       <c r="E23" s="12" t="n">
         <v>1</v>
@@ -3435,28 +3435,28 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Test sensors/servo signals before soldering. Kimi said optional; re-added because Hasan asked.</t>
+          <t>Must-have: check each power supply's voltage before plugging servos in (12 V by mistake burns 6 V servos).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Heat shrink</t>
+          <t>Breadboards + jumper wires</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>ASHINER heat shrink kit, 580 pcs</t>
+          <t>830 + 400 point breadboards with jumper wire kit</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B08XXGNJHG</t>
+          <t>https://www.amazon.ca/dp/B0BMFXPSVG</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
-        <v>14.99</v>
+        <v>19.99</v>
       </c>
       <c r="E24" s="12" t="n">
         <v>1</v>
@@ -3467,28 +3467,28 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Covers solder joints.</t>
+          <t>Test sensors/servo signals before soldering. Kimi said optional; re-added because Hasan asked.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>Calipers</t>
+          <t>Heat shrink</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ADORIC digital caliper 0-150 mm</t>
+          <t>ASHINER heat shrink kit, 580 pcs</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07DFFYCXS</t>
+          <t>https://www.amazon.ca/dp/B08XXGNJHG</t>
         </is>
       </c>
       <c r="D25" s="11" t="n">
-        <v>11.43</v>
+        <v>14.99</v>
       </c>
       <c r="E25" s="12" t="n">
         <v>1</v>
@@ -3499,28 +3499,28 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Measure screws and printed parts.</t>
+          <t>Covers solder joints.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Zip ties</t>
+          <t>Calipers</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>400 assorted zip ties</t>
+          <t>ADORIC digital caliper 0-150 mm</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B08TVLYB3Q</t>
+          <t>https://www.amazon.ca/dp/B07DFFYCXS</t>
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>11.98</v>
+        <v>11.43</v>
       </c>
       <c r="E26" s="12" t="n">
         <v>1</v>
@@ -3531,28 +3531,28 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Cable management.</t>
+          <t>Measure screws and printed parts.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Hot glue</t>
+          <t>Zip ties</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Surebonder LT-160 mini glue gun</t>
+          <t>400 assorted zip ties</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B004BPPHYE</t>
+          <t>https://www.amazon.ca/dp/B08TVLYB3Q</t>
         </is>
       </c>
       <c r="D27" s="11" t="n">
-        <v>7.47</v>
+        <v>11.98</v>
       </c>
       <c r="E27" s="12" t="n">
         <v>1</v>
@@ -3563,28 +3563,28 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>InMoov wire management method.</t>
+          <t>Cable management.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Needle files</t>
+          <t>Hot glue</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>10-piece needle file set</t>
+          <t>Surebonder LT-160 mini glue gun</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B07PPYWSCY</t>
+          <t>https://www.amazon.ca/dp/B004BPPHYE</t>
         </is>
       </c>
       <c r="D28" s="11" t="n">
-        <v>9.99</v>
+        <v>7.47</v>
       </c>
       <c r="E28" s="12" t="n">
         <v>1</v>
@@ -3595,28 +3595,28 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Fit printed parts (ball races, pistons). Kimi: day-1 blocker.</t>
+          <t>InMoov wire management method.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>Sandpaper</t>
+          <t>Needle files</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>3M sandpaper 100/150/220 grit, 5 sheets</t>
+          <t>10-piece needle file set</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B00004Z48U</t>
+          <t>https://www.amazon.ca/dp/B07PPYWSCY</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
-        <v>7.97</v>
+        <v>9.99</v>
       </c>
       <c r="E29" s="12" t="n">
         <v>1</v>
@@ -3627,28 +3627,28 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Smooth printed parts.</t>
+          <t>Fit printed parts (ball races, pistons). Kimi: day-1 blocker.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Hobby knife</t>
+          <t>Sandpaper</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>VViViD modelers knife + spare blades</t>
+          <t>3M sandpaper 100/150/220 grit, 5 sheets</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0CL5F9M4H</t>
+          <t>https://www.amazon.ca/dp/B00004Z48U</t>
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>7.98</v>
+        <v>7.97</v>
       </c>
       <c r="E30" s="12" t="n">
         <v>1</v>
@@ -3659,28 +3659,28 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>Clean up prints.</t>
+          <t>Smooth printed parts.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>Tweezers</t>
+          <t>Hobby knife</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>NARZ 4-piece tweezers</t>
+          <t>VViViD modelers knife + spare blades</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B09JLXKWB5</t>
+          <t>https://www.amazon.ca/dp/B0CL5F9M4H</t>
         </is>
       </c>
       <c r="D31" s="11" t="n">
-        <v>6.29</v>
+        <v>7.98</v>
       </c>
       <c r="E31" s="12" t="n">
         <v>1</v>
@@ -3691,28 +3691,28 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>Threading finger tendons.</t>
+          <t>Clean up prints.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>Safety glasses</t>
+          <t>Tweezers</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Clear safety glasses, 3-pack</t>
+          <t>NARZ 4-piece tweezers</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>https://www.amazon.ca/dp/B0F2JL22QN</t>
+          <t>https://www.amazon.ca/dp/B09JLXKWB5</t>
         </is>
       </c>
       <c r="D32" s="11" t="n">
-        <v>13.49</v>
+        <v>6.29</v>
       </c>
       <c r="E32" s="12" t="n">
         <v>1</v>
@@ -3723,30 +3723,46 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
+          <t>Threading finger tendons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Safety glasses</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Clear safety glasses, 3-pack</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ca/dp/B0F2JL22QN</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>13.49</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="13">
+        <f>D33*E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
           <t>For cutting, soldering, springs.</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>Subtotal (CAD, pre-tax)</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="16">
-        <f>SUM(F5:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="15" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>With HST 13%</t>
+          <t>Subtotal (CAD, pre-tax)</t>
         </is>
       </c>
       <c r="B34" s="15" t="n"/>
@@ -3754,15 +3770,31 @@
       <c r="D34" s="15" t="n"/>
       <c r="E34" s="15" t="n"/>
       <c r="F34" s="16">
-        <f>F33*1.13</f>
+        <f>SUM(F5:F33)</f>
         <v/>
       </c>
       <c r="G34" s="15" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>With HST 13%</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="15" t="n"/>
+      <c r="D35" s="15" t="n"/>
+      <c r="E35" s="15" t="n"/>
+      <c r="F35" s="16">
+        <f>F34*1.13</f>
+        <v/>
+      </c>
+      <c r="G35" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A35:E35"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
@@ -3793,6 +3825,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>